<commit_message>
se agregan cambios para la presentacion que sea realiza a equipo de sodimac.
</commit_message>
<xml_diff>
--- a/productos/productos.xlsx
+++ b/productos/productos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Desarrollo\IA\Proyectos\ai-lectura-documentos\productos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B0AD70D-70FB-4266-9644-F94BD52E7420}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{448E1F95-D933-4EC4-BCE5-EB6CB152EF28}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{A0B9DDF5-816D-43FB-9C22-015FF2201B46}"/>
   </bookViews>
@@ -497,7 +497,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:6" ht="58" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>110386466</v>
       </c>
@@ -507,7 +507,7 @@
       <c r="C2" t="s">
         <v>0</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" s="1" t="s">
         <v>1</v>
       </c>
       <c r="E2">
@@ -517,7 +517,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:6" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>110236243</v>
       </c>
@@ -527,7 +527,7 @@
       <c r="C3" t="s">
         <v>3</v>
       </c>
-      <c r="D3" t="s">
+      <c r="D3" s="1" t="s">
         <v>4</v>
       </c>
       <c r="E3">
@@ -567,7 +567,7 @@
       <c r="C5" t="s">
         <v>17</v>
       </c>
-      <c r="D5" t="s">
+      <c r="D5" s="1" t="s">
         <v>18</v>
       </c>
       <c r="E5">
@@ -577,7 +577,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:6" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A6">
         <v>143082664</v>
       </c>
@@ -587,7 +587,7 @@
       <c r="C6" t="s">
         <v>8</v>
       </c>
-      <c r="D6" t="s">
+      <c r="D6" s="1" t="s">
         <v>9</v>
       </c>
       <c r="E6">

</xml_diff>